<commit_message>
Sync Towards_SDS with edited master: AGE-DF rename, SCS-PI/TCS-AB/TCS-NK resolved
</commit_message>
<xml_diff>
--- a/terrestrial/Towards_SDS/Level4_SDS-aligned.xlsx
+++ b/terrestrial/Towards_SDS/Level4_SDS-aligned.xlsx
@@ -729,7 +729,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Argentina Distrito Federal</t>
+          <t>Ciudad Autónoma de Buenos Aires</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -742,18 +742,21 @@
           <t>AR</t>
         </is>
       </c>
-      <c r="F8" s="4" t="n"/>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H8" s="4" t="n"/>
       <c r="I8" s="4" t="n"/>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>AGE-DF (Argentina Distrito Federal) is integrated into AGE-BA. It is an incoherent disvision. Both are level 4 entities. Should AGE-DR be removed? 
-The toponym used for AGE-DR is not the most appropriate. The Autonomous City of Buenos Aires could have been used. http://www.infoleg.gob.ar/?page_id=166
+          <t>Ciudad Autónoma de Buenos Aires
 -Typographical error, where AGE-DR exists, there was AGE-DF. It is corrected according to TDWG.
 -AGE-DF It is not digitized on map 16 (pg 135)</t>
         </is>
@@ -17718,22 +17721,18 @@
           <t>SCS</t>
         </is>
       </c>
-      <c r="E511" s="4" t="inlineStr">
-        <is>
-          <t>PI*</t>
-        </is>
-      </c>
+      <c r="E511" s="4" t="n"/>
       <c r="F511" s="4" t="n"/>
       <c r="G511" s="4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H511" s="4" t="n"/>
       <c r="I511" s="4" t="n"/>
       <c r="J511" s="3" t="inlineStr">
         <is>
-          <t>The annotation must be included in the footer: "The PI* code  is adopted here unofficially for Paracel Is. though the ISO does not give them any code as their political status is disputed"</t>
+          <t>political status is disputed</t>
         </is>
       </c>
       <c r="K511" s="3" t="n"/>
@@ -19036,7 +19035,7 @@
       <c r="F549" s="4" t="n"/>
       <c r="G549" s="4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H549" s="4" t="inlineStr">
@@ -19250,7 +19249,7 @@
       <c r="F555" s="4" t="n"/>
       <c r="G555" s="4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H555" s="4" t="n"/>

</xml_diff>